<commit_message>
sample sheet changed. Formula removed from H7
</commit_message>
<xml_diff>
--- a/sequencing-app/NGS_sampleSheet_template.xlsx
+++ b/sequencing-app/NGS_sampleSheet_template.xlsx
@@ -1220,13 +1220,8 @@
       <c r="F4" s="31">
         <v>0.7</v>
       </c>
-      <c r="G4" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="42" t="str">
-        <f>A4&amp;"_"&amp;G4&amp;"_"&amp;B4</f>
-        <v>P1113_Sample01_30_F1</v>
-      </c>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
@@ -1247,13 +1242,8 @@
       <c r="F5" s="32">
         <v>0.1</v>
       </c>
-      <c r="G5" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="40" t="str">
-        <f>A5&amp;"_"&amp;G5&amp;"_"&amp;B5</f>
-        <v>P1113_Sample02_30_C1</v>
-      </c>
+      <c r="G5" s="39"/>
+      <c r="H5" s="40"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
@@ -1274,13 +1264,8 @@
       <c r="F6" s="32">
         <v>1.29</v>
       </c>
-      <c r="G6" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="40" t="str">
-        <f>A6&amp;"_"&amp;G6&amp;"_"&amp;B6</f>
-        <v>P1113_Sample03_1_F1</v>
-      </c>
+      <c r="G6" s="39"/>
+      <c r="H6" s="40"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="26" t="s">
@@ -1301,13 +1286,8 @@
       <c r="F7" s="33">
         <v>0.13</v>
       </c>
-      <c r="G7" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="44" t="str">
-        <f>A7&amp;"_"&amp;G7&amp;"_"&amp;B7</f>
-        <v>P1113_Sample04_1_C1</v>
-      </c>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
@@ -1526,13 +1506,8 @@
       <c r="D4" s="25"/>
       <c r="E4" s="35"/>
       <c r="F4" s="67"/>
-      <c r="G4" s="60" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="56" t="str">
-        <f>F4&amp;"_"&amp;G4&amp;"_"&amp;A4</f>
-        <v>_Sample01_</v>
-      </c>
+      <c r="G4" s="60"/>
+      <c r="H4" s="56"/>
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1542,13 +1517,8 @@
       <c r="D5" s="25"/>
       <c r="E5" s="35"/>
       <c r="F5" s="67"/>
-      <c r="G5" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="56" t="str">
-        <f>F5&amp;"_"&amp;G5&amp;"_"&amp;A5</f>
-        <v>_Sample02_</v>
-      </c>
+      <c r="G5" s="60"/>
+      <c r="H5" s="56"/>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1558,13 +1528,8 @@
       <c r="D6" s="25"/>
       <c r="E6" s="35"/>
       <c r="F6" s="67"/>
-      <c r="G6" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="56" t="str">
-        <f>F6&amp;"_"&amp;G6&amp;"_"&amp;A6</f>
-        <v>_Sample03_</v>
-      </c>
+      <c r="G6" s="60"/>
+      <c r="H6" s="56"/>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>